<commit_message>
Visualizacion de Ordenes Guardadas
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/INTORDENDECOMPRA.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/INTORDENDECOMPRA.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="16">
   <si>
     <t>CODIGO</t>
   </si>
@@ -90,6 +90,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -467,10 +468,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1658ADDC-DCFD-4FC0-A51D-94B360144F05}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.36328125" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -496,100 +497,326 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1357</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1357.0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1357.0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1357.0</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2">
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F4" t="n">
         <v>1771.62</v>
       </c>
-      <c r="G2">
-        <f>E2*F2</f>
-        <v>5314.86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>1357</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="G4" t="n">
+        <v>1771.62</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1357.0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1358.0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1771.62</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1771.62</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1358.0</v>
+      </c>
+      <c r="B7" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C7" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3" s="2">
-        <v>2137.5100000000002</v>
-      </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G5" si="0">E3*F3</f>
-        <v>8550.0400000000009</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>1357</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1358.0</v>
+      </c>
+      <c r="B8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C8" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4">
-        <v>5</v>
-      </c>
-      <c r="F4" s="2">
-        <v>2137.5100000000002</v>
-      </c>
-      <c r="G4">
-        <f t="shared" si="0"/>
-        <v>10687.550000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>1357</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1358.0</v>
+      </c>
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C9" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5" s="2">
-        <v>2137.5100000000002</v>
-      </c>
-      <c r="G5">
-        <f t="shared" si="0"/>
-        <v>12825.060000000001</v>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1359.0</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1771.62</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1771.62</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1359.0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1359.0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1359.0</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1360.0</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1360.0</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2137.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orden de Compra Finalizada
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/INTORDENDECOMPRA.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/INTORDENDECOMPRA.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80EFDD01-AD33-451A-9074-E63CA1AACFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6969066-96AB-4820-A30F-1BABC7517B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{92F47CF0-95F9-4D84-814C-7AFFA20164B6}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
   <si>
     <t>CODIGO</t>
   </si>
@@ -90,7 +90,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -126,14 +125,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,10 +461,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1658ADDC-DCFD-4FC0-A51D-94B360144F05}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.36328125" collapsed="true"/>
+    <col min="3" max="3" width="12.36328125" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -497,78 +490,78 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1357.0</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1771.62</v>
+      </c>
+      <c r="G2">
+        <v>1771.62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1357.0</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G3">
+        <v>2137.5100000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1357.0</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
       <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1771.62</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1771.62</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1357.0</v>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G4">
+        <v>2137.5100000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -579,19 +572,19 @@
       <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>1358.0</v>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G5">
+        <v>2137.5100000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -602,19 +595,19 @@
       <c r="D6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>1771.62</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>1771.62</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1358.0</v>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>3</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
@@ -625,19 +618,19 @@
       <c r="D7" t="s">
         <v>9</v>
       </c>
-      <c r="E7" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>1358.0</v>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G7">
+        <v>2137.5100000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>3</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
@@ -648,19 +641,19 @@
       <c r="D8" t="s">
         <v>9</v>
       </c>
-      <c r="E8" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>1358.0</v>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G8">
+        <v>2137.5100000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>3</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
@@ -671,19 +664,19 @@
       <c r="D9" t="s">
         <v>9</v>
       </c>
-      <c r="E9" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G9" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>1359.0</v>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G9">
+        <v>2137.5100000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>1</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -694,175 +687,37 @@
       <c r="D10" t="s">
         <v>9</v>
       </c>
-      <c r="E10" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F10" t="n">
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>1771.62</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>1771.62</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>1359.0</v>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
         <v>9</v>
       </c>
-      <c r="E11" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>1359.0</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G12" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>1359.0</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G13" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>1360.0</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G14" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>1360.0</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G15" t="n">
-        <v>2137.51</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>1361.0</v>
-      </c>
-      <c r="B16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1771.62</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1771.62</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>1361.0</v>
-      </c>
-      <c r="B17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>2137.51</v>
-      </c>
-      <c r="G17" t="n">
-        <v>2137.51</v>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>2137.5100000000002</v>
+      </c>
+      <c r="G11">
+        <v>2137.5100000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>